<commit_message>
Aggiornamento contenuti - 03/07/2026 14:22:09,21
</commit_message>
<xml_diff>
--- a/public/assets/03.Project/Projects List.xlsx
+++ b/public/assets/03.Project/Projects List.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MENTA\Desktop\GlemWebSite-main\public\assets\03.Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DBB6705-1496-46E0-8209-AF7BC818D582}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47C9CB08-5E49-4A88-A534-6B5959ED736B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31320" yWindow="1980" windowWidth="16095" windowHeight="12600" tabRatio="528" xr2:uid="{2E41E0B1-3E66-4403-8884-0B501731E142}"/>
+    <workbookView xWindow="28680" yWindow="690" windowWidth="19440" windowHeight="15000" tabRatio="528" xr2:uid="{2E41E0B1-3E66-4403-8884-0B501731E142}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="40">
   <si>
     <t>22.Lubica22-Y</t>
   </si>
@@ -65,9 +65,6 @@
     <t>25.MDW25-MiraProject</t>
   </si>
   <si>
-    <t>25MDW25-Metanoia</t>
-  </si>
-  <si>
     <t>Folder Name</t>
   </si>
   <si>
@@ -150,6 +147,18 @@
   </si>
   <si>
     <t>CLIMAX ad ArchiTexturExpo: da componente industriale a organismo architettonico | ATI Project</t>
+  </si>
+  <si>
+    <t>25.MDW25-Metanoia</t>
+  </si>
+  <si>
+    <t>25.ROMA-MicroMegaLAB</t>
+  </si>
+  <si>
+    <t>26.MDW26-KENOSIS</t>
+  </si>
+  <si>
+    <t>/KENOSIS: Lo svuotamento come atto generativo al Fuorisalone 2026 | ATI Project</t>
   </si>
 </sst>
 </file>
@@ -235,8 +244,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5D4E21C0-C8D9-4A0D-B0C1-DA6EEBC54DFD}" name="Tabella2" displayName="Tabella2" ref="A1:K38" totalsRowShown="0">
-  <autoFilter ref="A1:K38" xr:uid="{5D4E21C0-C8D9-4A0D-B0C1-DA6EEBC54DFD}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5D4E21C0-C8D9-4A0D-B0C1-DA6EEBC54DFD}" name="Tabella2" displayName="Tabella2" ref="A1:K39" totalsRowShown="0">
+  <autoFilter ref="A1:K39" xr:uid="{5D4E21C0-C8D9-4A0D-B0C1-DA6EEBC54DFD}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{9B3E0F3F-E2E3-49A1-9754-C0FF3F238018}" name="Folder Name"/>
     <tableColumn id="2" xr3:uid="{FACF951D-BE70-4A1B-99DB-5CE48A098CC2}" name="Link Article" dataDxfId="1"/>
@@ -571,7 +580,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFF62B37-38F8-4779-87AC-5A06A288B5EC}">
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38.140625" customWidth="1"/>
@@ -582,37 +591,37 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>10</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>11</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>12</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>13</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>14</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>15</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>16</v>
-      </c>
-      <c r="K1" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -620,11 +629,11 @@
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -632,11 +641,11 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -644,20 +653,20 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" t="s">
         <v>23</v>
       </c>
-      <c r="E4" t="s">
-        <v>24</v>
-      </c>
       <c r="F4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" t="s">
         <v>19</v>
-      </c>
-      <c r="G4" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -665,11 +674,11 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -677,13 +686,13 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="30" x14ac:dyDescent="0.25">
@@ -691,40 +700,35 @@
         <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E7" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>32</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" t="s">
         <v>23</v>
-      </c>
-      <c r="E8" t="s">
-        <v>24</v>
       </c>
       <c r="F8" t="s">
         <v>19</v>
       </c>
-      <c r="G8" t="s">
-        <v>20</v>
-      </c>
     </row>
     <row r="9" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>31</v>
@@ -733,35 +737,66 @@
       <c r="D9" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" t="s">
+        <v>18</v>
+      </c>
+      <c r="G9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>8</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="2"/>
       <c r="D10" t="s">
-        <v>23</v>
-      </c>
-      <c r="E10" t="s">
-        <v>24</v>
-      </c>
-      <c r="G10" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D11" t="s">
+      <c r="D12" t="s">
+        <v>21</v>
+      </c>
+      <c r="E12" t="s">
+        <v>23</v>
+      </c>
+      <c r="F12" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" t="s">
         <v>22</v>
       </c>
-      <c r="E11" t="s">
-        <v>24</v>
-      </c>
-      <c r="F11" t="s">
+      <c r="E13" t="s">
+        <v>23</v>
+      </c>
+      <c r="F13" t="s">
         <v>19</v>
       </c>
     </row>
@@ -770,18 +805,19 @@
   <hyperlinks>
     <hyperlink ref="B6" r:id="rId1" xr:uid="{BFE5A718-C745-4D4D-AA5B-43D9B2B73E47}"/>
     <hyperlink ref="B7" r:id="rId2" xr:uid="{C9311405-C9E4-497D-B9C4-EC5938A97AE0}"/>
-    <hyperlink ref="B8" r:id="rId3" xr:uid="{A72F001C-E42B-4EF8-857D-2FA7A4EB90BD}"/>
-    <hyperlink ref="B9" r:id="rId4" xr:uid="{7D3764A3-4CB9-403F-8BEB-D6CF6BDEE335}"/>
+    <hyperlink ref="B9" r:id="rId3" xr:uid="{A72F001C-E42B-4EF8-857D-2FA7A4EB90BD}"/>
+    <hyperlink ref="B10" r:id="rId4" xr:uid="{7D3764A3-4CB9-403F-8BEB-D6CF6BDEE335}"/>
     <hyperlink ref="B5" r:id="rId5" xr:uid="{7530A9CA-7CAF-45E2-A007-78A1B64F0B37}"/>
     <hyperlink ref="B4" r:id="rId6" xr:uid="{CA02230B-BF7E-4AE6-B0E8-6A124ABCA73B}"/>
     <hyperlink ref="B3" r:id="rId7" xr:uid="{E85E65DF-840C-4CF2-B4B3-91D673C45515}"/>
     <hyperlink ref="B2" r:id="rId8" xr:uid="{E9C9A097-FAEE-4A2C-B30F-20C43B06FB0A}"/>
     <hyperlink ref="C6" r:id="rId9" display="https://atiproject.com/attualita/design-temporariness-lucca-biennale-cartasia/" xr:uid="{43F23E5E-EE09-489E-9960-9EC8A8E3C1DE}"/>
-    <hyperlink ref="B11" r:id="rId10" display="https://atiproject.com/news/ati-project-climax-fuorisalone-2026/" xr:uid="{761E0EE4-767F-4188-A36D-524ECAD26F21}"/>
+    <hyperlink ref="B12" r:id="rId10" display="https://atiproject.com/news/ati-project-climax-fuorisalone-2026/" xr:uid="{761E0EE4-767F-4188-A36D-524ECAD26F21}"/>
+    <hyperlink ref="B13" r:id="rId11" display="https://atiproject.com/news/kenosis-fuorisalone-2026/" xr:uid="{521B91EE-5A7D-4965-8EFB-B74283953947}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId11"/>
+    <tablePart r:id="rId12"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>